<commit_message>
Fixes to fuel economy values for natural gas and LPG LDV passenger cars
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\BHNVFEAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49189A5-499E-4812-B686-83989CBCADAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6AA64CD-2303-4739-8481-1649E12569B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="19200" windowHeight="10050" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="43200" windowHeight="17145" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="110">
   <si>
     <t>Sources:</t>
   </si>
@@ -401,6 +401,18 @@
   </si>
   <si>
     <t>outputs read the SYFAFE tab, not the BNVFE tab.</t>
+  </si>
+  <si>
+    <t>Natural gas and LPG passenger LDV refresh (2026-09-25):</t>
+  </si>
+  <si>
+    <t>The internal 'BNVFE' tab's natural gas and LPG rows (rows 25 and 29, 2023-2050) are that tab's gasoline row times the CNG and LPG</t>
+  </si>
+  <si>
+    <t>fuel economy ratios to gasoline from the BNVFE workbook (calcs rows 113-114; NEMS AEO 2026 AFVADJFE = 1.00), because BNVFE had both</t>
+  </si>
+  <si>
+    <t>rows at 0 from 2023. The rest of that tab predates the 9a1e7ebf rebase of BNVFE, so its 2024-onward values differ from the current BNVFE.</t>
   </si>
 </sst>
 </file>
@@ -7806,11 +7818,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B56"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:B61"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.453125" customWidth="1"/>
-    <col min="2" max="2" width="107.453125" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="107.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -8051,6 +8063,26 @@
     <row r="56" spans="1:1">
       <c r="A56" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -8068,12 +8100,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -9062,13 +9094,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -9935,12 +9967,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -10807,14 +10839,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF13"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" customWidth="1"/>
-    <col min="3" max="3" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" spans="1:32" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -11708,12 +11740,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -12580,12 +12612,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -13566,12 +13598,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -14438,12 +14470,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -15432,12 +15464,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:31" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -16205,11 +16237,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AK30"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.453125" customWidth="1"/>
-    <col min="2" max="2" width="16.453125" customWidth="1"/>
-    <col min="3" max="3" width="30.7265625" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37">
@@ -17935,88 +17967,88 @@
         <v>4.1583860682125711E-4</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>4.0102815590911211E-4</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>3.7447643323240698E-4</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>3.9011286777709445E-4</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>3.973908333465341E-4</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>3.9921116827982341E-4</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>4.0474968459162865E-4</v>
       </c>
       <c r="J25">
-        <v>0</v>
+        <v>4.0866714086181205E-4</v>
       </c>
       <c r="K25">
-        <v>0</v>
+        <v>4.1165739618674141E-4</v>
       </c>
       <c r="L25">
-        <v>0</v>
+        <v>4.1453743818293512E-4</v>
       </c>
       <c r="M25">
-        <v>0</v>
+        <v>4.1476226395269379E-4</v>
       </c>
       <c r="N25">
-        <v>0</v>
+        <v>4.1467751199658729E-4</v>
       </c>
       <c r="O25">
-        <v>0</v>
+        <v>4.1774836203476703E-4</v>
       </c>
       <c r="P25">
-        <v>0</v>
+        <v>4.1834632264550211E-4</v>
       </c>
       <c r="Q25">
-        <v>0</v>
+        <v>4.1983822558637316E-4</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>4.2130104966706447E-4</v>
       </c>
       <c r="S25">
-        <v>0</v>
+        <v>4.2281184411175634E-4</v>
       </c>
       <c r="T25">
-        <v>0</v>
+        <v>4.2360951790740064E-4</v>
       </c>
       <c r="U25">
-        <v>0</v>
+        <v>4.2374431078237557E-4</v>
       </c>
       <c r="V25">
-        <v>0</v>
+        <v>4.2455978231601869E-4</v>
       </c>
       <c r="W25">
-        <v>0</v>
+        <v>4.2499271222158055E-4</v>
       </c>
       <c r="X25">
-        <v>0</v>
+        <v>4.255977010533903E-4</v>
       </c>
       <c r="Y25">
-        <v>0</v>
+        <v>4.259134403023234E-4</v>
       </c>
       <c r="Z25">
-        <v>0</v>
+        <v>4.2644140225411056E-4</v>
       </c>
       <c r="AA25">
-        <v>0</v>
+        <v>4.2668500307371869E-4</v>
       </c>
       <c r="AB25">
-        <v>0</v>
+        <v>4.2678409185942635E-4</v>
       </c>
       <c r="AC25">
-        <v>0</v>
+        <v>4.2712969246070032E-4</v>
       </c>
       <c r="AD25">
-        <v>0</v>
+        <v>4.274732939624897E-4</v>
       </c>
       <c r="AE25">
-        <v>0</v>
+        <v>4.2842378634895789E-4</v>
       </c>
     </row>
     <row r="26" spans="1:37">
@@ -18315,88 +18347,88 @@
         <v>3.5950684514816466E-4</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>4.0102815590911211E-4</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>3.7447643323240698E-4</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>3.9011286777709445E-4</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>3.973908333465341E-4</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>3.9921116827982341E-4</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>4.0474968459162865E-4</v>
       </c>
       <c r="J29">
-        <v>0</v>
+        <v>4.0866714086181205E-4</v>
       </c>
       <c r="K29">
-        <v>0</v>
+        <v>4.1165739618674141E-4</v>
       </c>
       <c r="L29">
-        <v>0</v>
+        <v>4.1453743818293512E-4</v>
       </c>
       <c r="M29">
-        <v>0</v>
+        <v>4.1476226395269379E-4</v>
       </c>
       <c r="N29">
-        <v>0</v>
+        <v>4.1467751199658729E-4</v>
       </c>
       <c r="O29">
-        <v>0</v>
+        <v>4.1774836203476703E-4</v>
       </c>
       <c r="P29">
-        <v>0</v>
+        <v>4.1834632264550211E-4</v>
       </c>
       <c r="Q29">
-        <v>0</v>
+        <v>4.1983822558637316E-4</v>
       </c>
       <c r="R29">
-        <v>0</v>
+        <v>4.2130104966706447E-4</v>
       </c>
       <c r="S29">
-        <v>0</v>
+        <v>4.2281184411175634E-4</v>
       </c>
       <c r="T29">
-        <v>0</v>
+        <v>4.2360951790740064E-4</v>
       </c>
       <c r="U29">
-        <v>0</v>
+        <v>4.2374431078237557E-4</v>
       </c>
       <c r="V29">
-        <v>0</v>
+        <v>4.2455978231601869E-4</v>
       </c>
       <c r="W29">
-        <v>0</v>
+        <v>4.2499271222158055E-4</v>
       </c>
       <c r="X29">
-        <v>0</v>
+        <v>4.255977010533903E-4</v>
       </c>
       <c r="Y29">
-        <v>0</v>
+        <v>4.259134403023234E-4</v>
       </c>
       <c r="Z29">
-        <v>0</v>
+        <v>4.2644140225411056E-4</v>
       </c>
       <c r="AA29">
-        <v>0</v>
+        <v>4.2668500307371869E-4</v>
       </c>
       <c r="AB29">
-        <v>0</v>
+        <v>4.2678409185942635E-4</v>
       </c>
       <c r="AC29">
-        <v>0</v>
+        <v>4.2712969246070032E-4</v>
       </c>
       <c r="AD29">
-        <v>0</v>
+        <v>4.274732939624897E-4</v>
       </c>
       <c r="AE29">
-        <v>0</v>
+        <v>4.2842378634895789E-4</v>
       </c>
     </row>
     <row r="30" spans="1:37">
@@ -18502,7 +18534,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
@@ -18876,9 +18908,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="50.453125" customWidth="1"/>
+    <col min="1" max="1" width="50.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -18980,11 +19012,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AL31"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42.1796875" customWidth="1"/>
-    <col min="2" max="2" width="26.453125" customWidth="1"/>
-    <col min="3" max="3" width="42.81640625" customWidth="1"/>
+    <col min="1" max="1" width="42.140625" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" customWidth="1"/>
+    <col min="3" max="3" width="42.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -19154,7 +19186,7 @@
         <v>5.76</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="29">
+    <row r="20" spans="1:4" ht="30">
       <c r="A20" s="9" t="s">
         <v>68</v>
       </c>
@@ -19172,7 +19204,7 @@
         <v>6.7042622950819668</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="29">
+    <row r="22" spans="1:4" ht="30">
       <c r="A22" s="9" t="s">
         <v>70</v>
       </c>
@@ -19258,10 +19290,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:BT15"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="15" max="15" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:72">
@@ -22705,12 +22737,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH10"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -22946,115 +22978,115 @@
       </c>
       <c r="D3" s="4">
         <f>BNVFE!D25*('BHNVFEAL-LDVs-psgr'!D$4/BNVFE!D$26)</f>
-        <v>0</v>
+        <v>3.2682328105658763E-4</v>
       </c>
       <c r="E3" s="4">
         <f>BNVFE!E25*('BHNVFEAL-LDVs-psgr'!E$4/BNVFE!E$26)</f>
-        <v>0</v>
+        <v>3.310144208647194E-4</v>
       </c>
       <c r="F3" s="4">
         <f>BNVFE!F25*('BHNVFEAL-LDVs-psgr'!F$4/BNVFE!F$26)</f>
-        <v>0</v>
+        <v>3.3520556067285118E-4</v>
       </c>
       <c r="G3" s="4">
         <f>BNVFE!G25*('BHNVFEAL-LDVs-psgr'!G$4/BNVFE!G$26)</f>
-        <v>0</v>
+        <v>3.3939670048098295E-4</v>
       </c>
       <c r="H3" s="4">
         <f>BNVFE!H25*('BHNVFEAL-LDVs-psgr'!H$4/BNVFE!H$26)</f>
-        <v>0</v>
+        <v>3.4358784028911473E-4</v>
       </c>
       <c r="I3" s="4">
         <f>BNVFE!I25*('BHNVFEAL-LDVs-psgr'!I$4/BNVFE!I$26)</f>
-        <v>0</v>
+        <v>3.477789800972465E-4</v>
       </c>
       <c r="J3" s="4">
         <f>BNVFE!J25*('BHNVFEAL-LDVs-psgr'!J$4/BNVFE!J$26)</f>
-        <v>0</v>
+        <v>3.5197011990537828E-4</v>
       </c>
       <c r="K3" s="4">
         <f>BNVFE!K25*('BHNVFEAL-LDVs-psgr'!K$4/BNVFE!K$26)</f>
-        <v>0</v>
+        <v>3.5616125971351005E-4</v>
       </c>
       <c r="L3" s="4">
         <f>BNVFE!L25*('BHNVFEAL-LDVs-psgr'!L$4/BNVFE!L$26)</f>
-        <v>0</v>
+        <v>3.6035239952164183E-4</v>
       </c>
       <c r="M3" s="4">
         <f>BNVFE!M25*('BHNVFEAL-LDVs-psgr'!M$4/BNVFE!M$26)</f>
-        <v>0</v>
+        <v>3.645435393297736E-4</v>
       </c>
       <c r="N3" s="4">
         <f>BNVFE!N25*('BHNVFEAL-LDVs-psgr'!N$4/BNVFE!N$26)</f>
-        <v>0</v>
+        <v>3.6873467913790537E-4</v>
       </c>
       <c r="O3" s="4">
         <f>BNVFE!O25*('BHNVFEAL-LDVs-psgr'!O$4/BNVFE!O$26)</f>
-        <v>0</v>
+        <v>3.7292581894603715E-4</v>
       </c>
       <c r="P3" s="4">
         <f>BNVFE!P25*('BHNVFEAL-LDVs-psgr'!P$4/BNVFE!P$26)</f>
-        <v>0</v>
+        <v>3.7711695875416892E-4</v>
       </c>
       <c r="Q3" s="4">
         <f>BNVFE!Q25*('BHNVFEAL-LDVs-psgr'!Q$4/BNVFE!Q$26)</f>
-        <v>0</v>
+        <v>3.813080985623007E-4</v>
       </c>
       <c r="R3" s="4">
         <f>BNVFE!R25*('BHNVFEAL-LDVs-psgr'!R$4/BNVFE!R$26)</f>
-        <v>0</v>
+        <v>3.8549923837043247E-4</v>
       </c>
       <c r="S3" s="4">
         <f>BNVFE!S25*('BHNVFEAL-LDVs-psgr'!S$4/BNVFE!S$26)</f>
-        <v>0</v>
+        <v>3.8969037817856381E-4</v>
       </c>
       <c r="T3" s="4">
         <f>BNVFE!T25*('BHNVFEAL-LDVs-psgr'!T$4/BNVFE!T$26)</f>
-        <v>0</v>
+        <v>3.9985001436006255E-4</v>
       </c>
       <c r="U3" s="4">
         <f>BNVFE!U25*('BHNVFEAL-LDVs-psgr'!U$4/BNVFE!U$26)</f>
-        <v>0</v>
+        <v>4.0645495978422236E-4</v>
       </c>
       <c r="V3" s="4">
         <f>BNVFE!V25*('BHNVFEAL-LDVs-psgr'!V$4/BNVFE!V$26)</f>
-        <v>0</v>
+        <v>4.1222868457836193E-4</v>
       </c>
       <c r="W3" s="4">
         <f>BNVFE!W25*('BHNVFEAL-LDVs-psgr'!W$4/BNVFE!W$26)</f>
-        <v>0</v>
+        <v>4.1315950014361388E-4</v>
       </c>
       <c r="X3" s="4">
         <f>BNVFE!X25*('BHNVFEAL-LDVs-psgr'!X$4/BNVFE!X$26)</f>
-        <v>0</v>
+        <v>4.1586031572729884E-4</v>
       </c>
       <c r="Y3" s="4">
         <f>BNVFE!Y25*('BHNVFEAL-LDVs-psgr'!Y$4/BNVFE!Y$26)</f>
-        <v>0</v>
+        <v>4.1791006177450995E-4</v>
       </c>
       <c r="Z3" s="4">
         <f>BNVFE!Z25*('BHNVFEAL-LDVs-psgr'!Z$4/BNVFE!Z$26)</f>
-        <v>0</v>
+        <v>4.1868747861134429E-4</v>
       </c>
       <c r="AA3" s="4">
         <f>BNVFE!AA25*('BHNVFEAL-LDVs-psgr'!AA$4/BNVFE!AA$26)</f>
-        <v>0</v>
+        <v>4.2132009406936789E-4</v>
       </c>
       <c r="AB3" s="4">
         <f>BNVFE!AB25*('BHNVFEAL-LDVs-psgr'!AB$4/BNVFE!AB$26)</f>
-        <v>0</v>
+        <v>4.224153063913546E-4</v>
       </c>
       <c r="AC3" s="4">
         <f>BNVFE!AC25*('BHNVFEAL-LDVs-psgr'!AC$4/BNVFE!AC$26)</f>
-        <v>0</v>
+        <v>4.2414977562549528E-4</v>
       </c>
       <c r="AD3" s="4">
         <f>BNVFE!AD25*('BHNVFEAL-LDVs-psgr'!AD$4/BNVFE!AD$26)</f>
-        <v>0</v>
+        <v>4.2551597947059568E-4</v>
       </c>
       <c r="AE3" s="4">
         <f>BNVFE!AE25*('BHNVFEAL-LDVs-psgr'!AE$4/BNVFE!AE$26)</f>
-        <v>0</v>
+        <v>4.2699017471707065E-4</v>
       </c>
       <c r="AG3" s="4"/>
       <c r="AH3" s="4"/>
@@ -23454,115 +23486,115 @@
       </c>
       <c r="D7" s="4">
         <f>BNVFE!D29*('BHNVFEAL-LDVs-psgr'!D$4/BNVFE!D$26)</f>
-        <v>0</v>
+        <v>3.2682328105658763E-4</v>
       </c>
       <c r="E7" s="4">
         <f>BNVFE!E29*('BHNVFEAL-LDVs-psgr'!E$4/BNVFE!E$26)</f>
-        <v>0</v>
+        <v>3.310144208647194E-4</v>
       </c>
       <c r="F7" s="4">
         <f>BNVFE!F29*('BHNVFEAL-LDVs-psgr'!F$4/BNVFE!F$26)</f>
-        <v>0</v>
+        <v>3.3520556067285118E-4</v>
       </c>
       <c r="G7" s="4">
         <f>BNVFE!G29*('BHNVFEAL-LDVs-psgr'!G$4/BNVFE!G$26)</f>
-        <v>0</v>
+        <v>3.3939670048098295E-4</v>
       </c>
       <c r="H7" s="4">
         <f>BNVFE!H29*('BHNVFEAL-LDVs-psgr'!H$4/BNVFE!H$26)</f>
-        <v>0</v>
+        <v>3.4358784028911473E-4</v>
       </c>
       <c r="I7" s="4">
         <f>BNVFE!I29*('BHNVFEAL-LDVs-psgr'!I$4/BNVFE!I$26)</f>
-        <v>0</v>
+        <v>3.477789800972465E-4</v>
       </c>
       <c r="J7" s="4">
         <f>BNVFE!J29*('BHNVFEAL-LDVs-psgr'!J$4/BNVFE!J$26)</f>
-        <v>0</v>
+        <v>3.5197011990537828E-4</v>
       </c>
       <c r="K7" s="4">
         <f>BNVFE!K29*('BHNVFEAL-LDVs-psgr'!K$4/BNVFE!K$26)</f>
-        <v>0</v>
+        <v>3.5616125971351005E-4</v>
       </c>
       <c r="L7" s="4">
         <f>BNVFE!L29*('BHNVFEAL-LDVs-psgr'!L$4/BNVFE!L$26)</f>
-        <v>0</v>
+        <v>3.6035239952164183E-4</v>
       </c>
       <c r="M7" s="4">
         <f>BNVFE!M29*('BHNVFEAL-LDVs-psgr'!M$4/BNVFE!M$26)</f>
-        <v>0</v>
+        <v>3.645435393297736E-4</v>
       </c>
       <c r="N7" s="4">
         <f>BNVFE!N29*('BHNVFEAL-LDVs-psgr'!N$4/BNVFE!N$26)</f>
-        <v>0</v>
+        <v>3.6873467913790537E-4</v>
       </c>
       <c r="O7" s="4">
         <f>BNVFE!O29*('BHNVFEAL-LDVs-psgr'!O$4/BNVFE!O$26)</f>
-        <v>0</v>
+        <v>3.7292581894603715E-4</v>
       </c>
       <c r="P7" s="4">
         <f>BNVFE!P29*('BHNVFEAL-LDVs-psgr'!P$4/BNVFE!P$26)</f>
-        <v>0</v>
+        <v>3.7711695875416892E-4</v>
       </c>
       <c r="Q7" s="4">
         <f>BNVFE!Q29*('BHNVFEAL-LDVs-psgr'!Q$4/BNVFE!Q$26)</f>
-        <v>0</v>
+        <v>3.813080985623007E-4</v>
       </c>
       <c r="R7" s="4">
         <f>BNVFE!R29*('BHNVFEAL-LDVs-psgr'!R$4/BNVFE!R$26)</f>
-        <v>0</v>
+        <v>3.8549923837043247E-4</v>
       </c>
       <c r="S7" s="4">
         <f>BNVFE!S29*('BHNVFEAL-LDVs-psgr'!S$4/BNVFE!S$26)</f>
-        <v>0</v>
+        <v>3.8969037817856381E-4</v>
       </c>
       <c r="T7" s="4">
         <f>BNVFE!T29*('BHNVFEAL-LDVs-psgr'!T$4/BNVFE!T$26)</f>
-        <v>0</v>
+        <v>3.9985001436006255E-4</v>
       </c>
       <c r="U7" s="4">
         <f>BNVFE!U29*('BHNVFEAL-LDVs-psgr'!U$4/BNVFE!U$26)</f>
-        <v>0</v>
+        <v>4.0645495978422236E-4</v>
       </c>
       <c r="V7" s="4">
         <f>BNVFE!V29*('BHNVFEAL-LDVs-psgr'!V$4/BNVFE!V$26)</f>
-        <v>0</v>
+        <v>4.1222868457836193E-4</v>
       </c>
       <c r="W7" s="4">
         <f>BNVFE!W29*('BHNVFEAL-LDVs-psgr'!W$4/BNVFE!W$26)</f>
-        <v>0</v>
+        <v>4.1315950014361388E-4</v>
       </c>
       <c r="X7" s="4">
         <f>BNVFE!X29*('BHNVFEAL-LDVs-psgr'!X$4/BNVFE!X$26)</f>
-        <v>0</v>
+        <v>4.1586031572729884E-4</v>
       </c>
       <c r="Y7" s="4">
         <f>BNVFE!Y29*('BHNVFEAL-LDVs-psgr'!Y$4/BNVFE!Y$26)</f>
-        <v>0</v>
+        <v>4.1791006177450995E-4</v>
       </c>
       <c r="Z7" s="4">
         <f>BNVFE!Z29*('BHNVFEAL-LDVs-psgr'!Z$4/BNVFE!Z$26)</f>
-        <v>0</v>
+        <v>4.1868747861134429E-4</v>
       </c>
       <c r="AA7" s="4">
         <f>BNVFE!AA29*('BHNVFEAL-LDVs-psgr'!AA$4/BNVFE!AA$26)</f>
-        <v>0</v>
+        <v>4.2132009406936789E-4</v>
       </c>
       <c r="AB7" s="4">
         <f>BNVFE!AB29*('BHNVFEAL-LDVs-psgr'!AB$4/BNVFE!AB$26)</f>
-        <v>0</v>
+        <v>4.224153063913546E-4</v>
       </c>
       <c r="AC7" s="4">
         <f>BNVFE!AC29*('BHNVFEAL-LDVs-psgr'!AC$4/BNVFE!AC$26)</f>
-        <v>0</v>
+        <v>4.2414977562549528E-4</v>
       </c>
       <c r="AD7" s="4">
         <f>BNVFE!AD29*('BHNVFEAL-LDVs-psgr'!AD$4/BNVFE!AD$26)</f>
-        <v>0</v>
+        <v>4.2551597947059568E-4</v>
       </c>
       <c r="AE7" s="4">
         <f>BNVFE!AE29*('BHNVFEAL-LDVs-psgr'!AE$4/BNVFE!AE$26)</f>
-        <v>0</v>
+        <v>4.2699017471707065E-4</v>
       </c>
       <c r="AG7" s="4"/>
       <c r="AH7" s="4"/>
@@ -23739,12 +23771,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -24733,12 +24765,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:34" ht="30">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>

</xml_diff>